<commit_message>
More cart test cases
</commit_message>
<xml_diff>
--- a/test_cases.xlsx
+++ b/test_cases.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Programming\Python\QA_Testing\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56051333-4387-4FDF-88BA-5DB7C4E59E9B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A13E6D24-BA14-4038-9D2B-E830DB9B577B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{8FBF4EF6-23A4-453E-A09F-460DDE2B30EF}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="105">
   <si>
     <t>ID</t>
   </si>
@@ -99,39 +99,7 @@
     <t>Step-by-Step Instructions</t>
   </si>
   <si>
-    <t>Clean browser instance
-Internet connection
-The email is not already used
-User is on the register page</t>
-  </si>
-  <si>
-    <t>Clean browser instance
-Internet connection
-User is on the register page</t>
-  </si>
-  <si>
-    <t>Internet connection
-Clean browser instance
-User is on login page</t>
-  </si>
-  <si>
-    <t>Internet connection
-Clean browser instance
-Current account was registered
-User is on login page</t>
-  </si>
-  <si>
     <t>OCD_Login_003</t>
-  </si>
-  <si>
-    <t>Internet connection
-Clean browser instance
-User is on home page</t>
-  </si>
-  <si>
-    <t>Internet connection
-Clean browser instance
-User is on any page</t>
   </si>
   <si>
     <t>1. user enters first name, last name, email, phone number, password, confirmed password
@@ -268,12 +236,6 @@
 3. user clicks 'Login' button</t>
   </si>
   <si>
-    <t>Internet connection
-Clean browser instance
-User is on any page
-4 'Mac' products are present in the db</t>
-  </si>
-  <si>
     <t>1. user enters "Mac" in the search bar on top
 2. clicks the 'Search' button</t>
   </si>
@@ -294,32 +256,12 @@
   <si>
     <t>1. user scrolls to the first product on home page
 2. clicks the 'Add to Cart' button</t>
-  </si>
-  <si>
-    <t>cart status should update on the right-top side</t>
   </si>
   <si>
     <t xml:space="preserve">1. user enters "mac" and presses 'Enter' in the search bar
 2. adds "iMac" to cart
 3. adds "MacBook Air" to cart
 </t>
-  </si>
-  <si>
-    <t>user should see cart status "2 item(s) - $1,324.00"</t>
-  </si>
-  <si>
-    <t>Internet connection
-Clean browser instance
-User in on home page</t>
-  </si>
-  <si>
-    <t>1. user enters "samsung" and presses 'Enter' in the search bar
-2. adds product "Samsung SyncMaster 941BW" to cart
-4. clicks cart icon
-3. deletes "Samsung SyncMaster 941BW" from cart</t>
-  </si>
-  <si>
-    <t>user can see empty cart</t>
   </si>
   <si>
     <t>Title</t>
@@ -361,6 +303,117 @@
   </si>
   <si>
     <t>Low</t>
+  </si>
+  <si>
+    <t>1. user enters "samsung" and presses 'Enter' in the search bar
+2. adds product "Samsung SyncMaster 941BW" to cart
+3. clicks cart icon
+4. deletes "Samsung SyncMaster 941BW" from cart</t>
+  </si>
+  <si>
+    <t>OCD_Cart_004</t>
+  </si>
+  <si>
+    <t>Product count update</t>
+  </si>
+  <si>
+    <t>User is on cart page
+Al least 1 product is in the cart</t>
+  </si>
+  <si>
+    <t>The email is not already used
+User is on the register page</t>
+  </si>
+  <si>
+    <t>User is on the register page</t>
+  </si>
+  <si>
+    <t>Current account was registered
+User is on login page</t>
+  </si>
+  <si>
+    <t>User is on login page</t>
+  </si>
+  <si>
+    <t>User is on any page
+4 'Mac' products are present in the db</t>
+  </si>
+  <si>
+    <t>User is on any page</t>
+  </si>
+  <si>
+    <t>User is on home page</t>
+  </si>
+  <si>
+    <t>User in on home page</t>
+  </si>
+  <si>
+    <t>cart item count updates to 1</t>
+  </si>
+  <si>
+    <t>cart item count updates to 2</t>
+  </si>
+  <si>
+    <t>cart is empty</t>
+  </si>
+  <si>
+    <t>1. on the first product user clicks the 'Quantity' input
+2. user types '3'
+3. user clicks the Update icon (button)</t>
+  </si>
+  <si>
+    <t>1. Qantity of product updates to '3'
+2. Update confirmation popup is visible
+3. Product subtotal cost updates
+4. Cart total cost updates</t>
+  </si>
+  <si>
+    <t>OCD_Cart_005</t>
+  </si>
+  <si>
+    <t>Inventory limits exceeded</t>
+  </si>
+  <si>
+    <t>User is on cart page
+'iMac' product is in cart</t>
+  </si>
+  <si>
+    <t>1. on 'iMac' product from cart user clicks 'Quantity' input
+2. user types '1000'
+3. user clicks the Update icon (button)</t>
+  </si>
+  <si>
+    <t>1. Errors is shown: "Products marked with *** are not available in the desired quantity or not in stock!"
+2. Product name changes to "iMac ***"</t>
+  </si>
+  <si>
+    <t>OCD_Cart_006</t>
+  </si>
+  <si>
+    <t>Cart persistance</t>
+  </si>
+  <si>
+    <t>1. user enters 'samsung' and presses 'Enter' in the search bar
+2. adds product "Samsung SyncMaster 941BW" to cart
+3. user logs out of account
+4. user logs back in</t>
+  </si>
+  <si>
+    <t>1. Cart item count is 1
+2. Product found in cart is "Samsung SyncMaster 941BW"</t>
+  </si>
+  <si>
+    <t>OCD_Cart_007</t>
+  </si>
+  <si>
+    <t>Cart empty by default</t>
+  </si>
+  <si>
+    <t>1. user clicks cart button</t>
+  </si>
+  <si>
+    <t>1. cart is empty
+2. 'Checkout' and 'View Cart' buttons are not visible</t>
   </si>
 </sst>
 </file>
@@ -396,9 +449,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -735,7 +794,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{80A021F8-77F7-49B4-AF4C-68F5356311C2}">
-  <dimension ref="A1:G16"/>
+  <dimension ref="A1:G20"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="23.7109375" customWidth="1"/>
@@ -750,7 +809,7 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="C1" t="s">
         <v>16</v>
@@ -765,7 +824,7 @@
         <v>3</v>
       </c>
       <c r="G1" t="s">
-        <v>85</v>
+        <v>73</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="75" x14ac:dyDescent="0.25">
@@ -773,16 +832,16 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>19</v>
+        <v>79</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>44</v>
+        <v>38</v>
       </c>
       <c r="F2">
         <v>1</v>
@@ -796,16 +855,16 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>20</v>
+        <v>80</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="F3">
         <v>2</v>
@@ -819,16 +878,16 @@
         <v>5</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>20</v>
+        <v>80</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="F4">
         <v>2</v>
@@ -837,21 +896,21 @@
         <v>15</v>
       </c>
     </row>
-    <row r="5" spans="1:7" ht="60" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" ht="45" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>7</v>
       </c>
       <c r="B5" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>22</v>
+        <v>81</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="E5" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="F5">
         <v>1</v>
@@ -860,21 +919,21 @@
         <v>15</v>
       </c>
     </row>
-    <row r="6" spans="1:7" ht="60" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" ht="45" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>6</v>
       </c>
       <c r="B6" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>22</v>
+        <v>81</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="F6">
         <v>3</v>
@@ -885,19 +944,19 @@
     </row>
     <row r="7" spans="1:7" ht="60" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>22</v>
+        <v>81</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="F7">
         <v>2</v>
@@ -908,19 +967,19 @@
     </row>
     <row r="8" spans="1:7" ht="45" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="B8" t="s">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>21</v>
+        <v>82</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="F8">
         <v>2</v>
@@ -929,44 +988,44 @@
         <v>4</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="60" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>62</v>
+        <v>83</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>65</v>
+        <v>58</v>
       </c>
       <c r="E9" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="F9">
         <v>3</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" ht="60" x14ac:dyDescent="0.25">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>10</v>
       </c>
       <c r="B10" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>62</v>
+        <v>83</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>63</v>
+        <v>56</v>
       </c>
       <c r="E10" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="F10">
         <v>1</v>
@@ -975,47 +1034,47 @@
         <v>4</v>
       </c>
     </row>
-    <row r="11" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>11</v>
       </c>
       <c r="B11" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>25</v>
+        <v>84</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>66</v>
+        <v>59</v>
       </c>
       <c r="E11" t="s">
-        <v>67</v>
+        <v>60</v>
       </c>
       <c r="F11">
         <v>3</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>12</v>
       </c>
       <c r="B12" t="s">
-        <v>37</v>
+        <v>31</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>24</v>
+        <v>85</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>68</v>
+        <v>61</v>
       </c>
       <c r="E12" t="s">
-        <v>69</v>
+        <v>87</v>
       </c>
       <c r="F12">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G12" s="1" t="s">
         <v>15</v>
@@ -1026,22 +1085,22 @@
         <v>13</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>24</v>
+        <v>85</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>70</v>
+        <v>62</v>
       </c>
       <c r="E13" t="s">
-        <v>71</v>
+        <v>88</v>
       </c>
       <c r="F13">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G13" s="1" t="s">
-        <v>86</v>
+        <v>4</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="60" x14ac:dyDescent="0.25">
@@ -1049,16 +1108,16 @@
         <v>14</v>
       </c>
       <c r="B14" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>72</v>
+        <v>86</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="E14" t="s">
-        <v>74</v>
+        <v>89</v>
       </c>
       <c r="F14">
         <v>3</v>
@@ -1067,49 +1126,141 @@
         <v>9</v>
       </c>
     </row>
-    <row r="15" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" ht="60" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>27</v>
-      </c>
-      <c r="B15" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="B15" t="s">
+        <v>77</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="F15">
+        <v>3</v>
+      </c>
+      <c r="G15" s="1" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>92</v>
+      </c>
+      <c r="B16" t="s">
+        <v>93</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="F16">
+        <v>2</v>
+      </c>
+      <c r="G16" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" ht="60" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>97</v>
+      </c>
+      <c r="B17" t="s">
+        <v>98</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="E17" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="F17">
+        <v>3</v>
+      </c>
+      <c r="G17" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>101</v>
+      </c>
+      <c r="B18" t="s">
+        <v>102</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="E18" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="F18">
+        <v>2</v>
+      </c>
+      <c r="G18" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>21</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="E19" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="C15" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="D15" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="E15" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="F15" s="1">
+      <c r="F19" s="1">
         <v>2</v>
       </c>
-      <c r="G15" s="1" t="s">
+      <c r="G19" s="1" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="16" spans="1:7" ht="30" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>48</v>
-      </c>
-      <c r="B16" t="s">
-        <v>49</v>
-      </c>
-      <c r="C16" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="D16" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="E16" t="s">
-        <v>52</v>
-      </c>
-      <c r="F16">
+    <row r="20" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>42</v>
+      </c>
+      <c r="B20" t="s">
+        <v>43</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="D20" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="E20" t="s">
+        <v>46</v>
+      </c>
+      <c r="F20">
         <v>1</v>
       </c>
-      <c r="G16" s="1" t="s">
+      <c r="G20" s="1" t="s">
         <v>15</v>
       </c>
     </row>
@@ -1129,42 +1280,42 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>75</v>
+        <v>63</v>
       </c>
       <c r="B1" t="s">
-        <v>80</v>
+        <v>68</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>76</v>
+        <v>64</v>
       </c>
       <c r="B2" t="s">
-        <v>81</v>
+        <v>69</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>77</v>
+        <v>65</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>82</v>
+        <v>70</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>78</v>
+        <v>66</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>83</v>
+        <v>71</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>79</v>
+        <v>67</v>
       </c>
       <c r="B5" t="s">
-        <v>84</v>
+        <v>72</v>
       </c>
     </row>
   </sheetData>

</xml_diff>